<commit_message>
Auto update: 2026-07-26 coffee data
</commit_message>
<xml_diff>
--- a/咖啡豆每日价格.xlsx
+++ b/咖啡豆每日价格.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1999,6 +1999,40 @@
         <v>#N/A</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>32.38</v>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>31.39</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="F46" s="2" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>26.14</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>24.18</v>
+      </c>
+      <c r="J46" s="2" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>